<commit_message>
Stage SHA-pinned ADAA public-safe refreshed candidate for Draft PR review
</commit_message>
<xml_diff>
--- a/public/assets/systems/adaa/ADAA_Portfolio_Target_History.xlsx
+++ b/public/assets/systems/adaa/ADAA_Portfolio_Target_History.xlsx
@@ -219,7 +219,7 @@
         <v>0.120833333333333</v>
       </c>
       <c r="E2" s="1">
-        <v>0.102083333333333</v>
+        <v>0.0729166666666667</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
@@ -267,7 +267,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.408333333333333</v>
+        <v>0.4375</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Publish SHA-pinned ADAA 2026-10-12 Pages canary data-only refresh
Co-authored-by: github-actions[bot] <41898282+github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/assets/systems/adaa/ADAA_Portfolio_Target_History.xlsx
+++ b/public/assets/systems/adaa/ADAA_Portfolio_Target_History.xlsx
@@ -219,7 +219,7 @@
         <v>0.120833333333333</v>
       </c>
       <c r="E2" s="1">
-        <v>0.102083333333333</v>
+        <v>0.0729166666666667</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
@@ -267,7 +267,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.408333333333333</v>
+        <v>0.4375</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
test: ADAA 2026-10-09 Pages-only recovery candidate (NEVER MERGE)
</commit_message>
<xml_diff>
--- a/public/assets/systems/adaa/ADAA_Portfolio_Target_History.xlsx
+++ b/public/assets/systems/adaa/ADAA_Portfolio_Target_History.xlsx
@@ -219,7 +219,7 @@
         <v>0.120833333333333</v>
       </c>
       <c r="E2" s="1">
-        <v>0.0729166666666667</v>
+        <v>0.102083333333333</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
@@ -267,7 +267,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>0.4375</v>
+        <v>0.408333333333333</v>
       </c>
     </row>
     <row r="3">

</xml_diff>